<commit_message>
fix: unify template empty rows and export border styles
</commit_message>
<xml_diff>
--- a/public/SO_THEO_DOI_TEMPLATE.xlsx
+++ b/public/SO_THEO_DOI_TEMPLATE.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="2" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="23">
   <si>
     <t/>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>Nhập/Xuất hàng</t>
-  </si>
-  <si>
-    <t>Ghi chú</t>
   </si>
   <si>
     <t>Giờ</t>
@@ -116,7 +113,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -176,13 +173,6 @@
       <sz val="11"/>
       <name val="Times New Roman"/>
     </font>
-    <font>
-      <charset val="163"/>
-      <color theme="1"/>
-      <family val="1"/>
-      <sz val="22"/>
-      <name val="Times New Roman"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -232,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -261,11 +251,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="6"/>
@@ -602,17 +595,20 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" ht="14.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" ht="14.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -627,7 +623,7 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
     </row>
-    <row r="3" ht="14.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" ht="14.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -642,13 +638,15 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" ht="14.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" ht="14.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>0</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -657,14 +655,17 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" ht="27.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E5" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="27.75" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
@@ -679,13 +680,15 @@
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
     </row>
-    <row r="7" ht="17.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" ht="17.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E7" s="6"/>
+      <c r="E7" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -704,59 +707,61 @@
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="9" t="s">
         <v>7</v>
-      </c>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="9" ht="41.25" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="K9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="L9" s="8"/>
-    </row>
-    <row r="10" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L9" s="9"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E10" s="10"/>
+      <c r="E10" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
@@ -765,13 +770,15 @@
       <c r="K10" s="10"/>
       <c r="L10" s="10"/>
     </row>
-    <row r="11" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E11" s="10"/>
+      <c r="E11" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
@@ -780,13 +787,15 @@
       <c r="K11" s="10"/>
       <c r="L11" s="10"/>
     </row>
-    <row r="12" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E12" s="10"/>
+      <c r="E12" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
@@ -795,13 +804,15 @@
       <c r="K12" s="10"/>
       <c r="L12" s="10"/>
     </row>
-    <row r="13" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
@@ -810,13 +821,15 @@
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
     </row>
-    <row r="14" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="10"/>
+      <c r="E14" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
@@ -825,13 +838,15 @@
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
     </row>
-    <row r="15" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="10"/>
+      <c r="E15" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
@@ -840,13 +855,15 @@
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
     </row>
-    <row r="16" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E16" s="10"/>
+      <c r="E16" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
@@ -855,13 +872,15 @@
       <c r="K16" s="10"/>
       <c r="L16" s="10"/>
     </row>
-    <row r="17" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E17" s="10"/>
+      <c r="E17" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
@@ -870,13 +889,15 @@
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
     </row>
-    <row r="18" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
@@ -885,13 +906,15 @@
       <c r="K18" s="10"/>
       <c r="L18" s="10"/>
     </row>
-    <row r="19" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
@@ -900,13 +923,15 @@
       <c r="K19" s="10"/>
       <c r="L19" s="10"/>
     </row>
-    <row r="20" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E20" s="10"/>
+      <c r="E20" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
@@ -915,13 +940,15 @@
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
     </row>
-    <row r="21" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E21" s="10"/>
+      <c r="E21" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
@@ -930,13 +957,15 @@
       <c r="K21" s="10"/>
       <c r="L21" s="10"/>
     </row>
-    <row r="22" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E22" s="10"/>
+      <c r="E22" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
@@ -945,13 +974,15 @@
       <c r="K22" s="10"/>
       <c r="L22" s="10"/>
     </row>
-    <row r="23" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E23" s="10"/>
+      <c r="E23" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
@@ -960,13 +991,15 @@
       <c r="K23" s="10"/>
       <c r="L23" s="10"/>
     </row>
-    <row r="24" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E24" s="10"/>
+      <c r="E24" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
@@ -975,13 +1008,15 @@
       <c r="K24" s="10"/>
       <c r="L24" s="10"/>
     </row>
-    <row r="25" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E25" s="10"/>
+      <c r="E25" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
@@ -990,13 +1025,15 @@
       <c r="K25" s="10"/>
       <c r="L25" s="10"/>
     </row>
-    <row r="26" ht="28.2" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="E26" s="10"/>
+      <c r="E26" s="10" t="s">
+        <v>0</v>
+      </c>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
@@ -1005,57 +1042,86 @@
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="11"/>
-      <c r="D27" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C27" s="11"/>
+      <c r="D27" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="10"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" t="s">
+        <v>0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D28" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B29" s="12" t="s">
+      <c r="D29" t="s">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D29" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="12" t="s">
+      <c r="D30" t="s">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D30" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="12" t="s">
+      <c r="D31" t="s">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D31" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B32" s="12" t="s">
+      <c r="D32" t="s">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D32" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="12" t="s">
-        <v>23</v>
-      </c>
       <c r="D33" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve header and data shifting on row 27 onwards, refine column widths
</commit_message>
<xml_diff>
--- a/public/SO_THEO_DOI_TEMPLATE.xlsx
+++ b/public/SO_THEO_DOI_TEMPLATE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="24">
   <si>
     <t/>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>Nhập/Xuất hàng</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
   </si>
   <si>
     <t>Giờ</t>
@@ -222,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -252,13 +255,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="6"/>
@@ -600,7 +606,7 @@
   <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
         <v>0</v>
       </c>
@@ -608,7 +614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="14.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="2" ht="14.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -623,7 +629,7 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
     </row>
-    <row r="3" ht="14.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" ht="14.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -638,7 +644,7 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" ht="14.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="4" ht="14.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
@@ -655,7 +661,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
@@ -665,7 +671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="27.75" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" ht="27.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
@@ -680,7 +686,7 @@
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
     </row>
-    <row r="7" ht="17.4" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" ht="17.4" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
@@ -707,53 +713,53 @@
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
       <c r="L8" s="9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" ht="41.25" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10" t="s">
@@ -762,15 +768,15 @@
       <c r="E10" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J10" s="12"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="12"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="10" t="s">
@@ -779,15 +785,15 @@
       <c r="E11" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
       <c r="H11" s="10"/>
       <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J11" s="12"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="12"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10" t="s">
@@ -796,15 +802,15 @@
       <c r="E12" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J12" s="12"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="12"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
@@ -813,15 +819,15 @@
       <c r="E13" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
       <c r="H13" s="10"/>
       <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J13" s="12"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="12"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10" t="s">
@@ -830,15 +836,15 @@
       <c r="E14" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J14" s="12"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="12"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10" t="s">
@@ -847,15 +853,15 @@
       <c r="E15" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J15" s="12"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="12"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10" t="s">
@@ -864,15 +870,15 @@
       <c r="E16" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J16" s="12"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="12"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10" t="s">
@@ -881,15 +887,15 @@
       <c r="E17" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J17" s="12"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="12"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10" t="s">
@@ -898,15 +904,15 @@
       <c r="E18" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
       <c r="H18" s="10"/>
       <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J18" s="12"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="12"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10" t="s">
@@ -915,15 +921,15 @@
       <c r="E19" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J19" s="12"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="12"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10" t="s">
@@ -932,15 +938,15 @@
       <c r="E20" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J20" s="12"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="12"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10" t="s">
@@ -949,15 +955,15 @@
       <c r="E21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
       <c r="H21" s="10"/>
       <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J21" s="12"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="12"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10" t="s">
@@ -966,15 +972,15 @@
       <c r="E22" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J22" s="12"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="12"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10" t="s">
@@ -983,15 +989,15 @@
       <c r="E23" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J23" s="12"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="12"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10" t="s">
@@ -1000,15 +1006,15 @@
       <c r="E24" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="10"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J24" s="12"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="12"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10" t="s">
@@ -1017,15 +1023,15 @@
       <c r="E25" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
       <c r="H25" s="10"/>
       <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J25" s="12"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="12"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10" t="s">
@@ -1034,34 +1040,34 @@
       <c r="E26" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
       <c r="H26" s="10"/>
       <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="10"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="11" t="s">
-        <v>17</v>
+      <c r="J26" s="12"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="12"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="12"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="13" t="s">
+        <v>18</v>
       </c>
       <c r="D28" t="s">
         <v>0</v>
@@ -1070,9 +1076,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" s="13" t="s">
-        <v>18</v>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="14" t="s">
+        <v>19</v>
       </c>
       <c r="D29" t="s">
         <v>0</v>
@@ -1081,9 +1087,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30" s="13" t="s">
-        <v>19</v>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="14" t="s">
+        <v>20</v>
       </c>
       <c r="D30" t="s">
         <v>0</v>
@@ -1092,9 +1098,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31" s="13" t="s">
-        <v>20</v>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="14" t="s">
+        <v>21</v>
       </c>
       <c r="D31" t="s">
         <v>0</v>
@@ -1103,9 +1109,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="13" t="s">
-        <v>21</v>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="14" t="s">
+        <v>22</v>
       </c>
       <c r="D32" t="s">
         <v>0</v>
@@ -1114,9 +1120,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="13" t="s">
-        <v>22</v>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B33" s="14" t="s">
+        <v>23</v>
       </c>
       <c r="D33" t="s">
         <v>0</v>

</xml_diff>